<commit_message>
Figure labels and supplement wording after the control review
- analysis/figures.py: Figure 2 labels the shaded band "transition interval",
  as the paper does; Figure 4 names the paired-design procedure "Original search".
- results/Supplementary_Tables_S1-S6.xlsx: "measurement kit of configuration D"
  instead of "revision kit" (sheet S5 and README); values unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GhxqJjDYH8jxjDNPcEyfRE
</commit_message>
<xml_diff>
--- a/results/Supplementary_Tables_S1-S6.xlsx
+++ b/results/Supplementary_Tables_S1-S6.xlsx
@@ -49,7 +49,7 @@
     <t xml:space="preserve">S4_NIST — NIST SP 800-22 results (100 bitstreams of 10^6 bits per sequence): for every test (and every template, excursion state, or variant), the number of passing bitstreams and the P-value of the uniformity test. Sequences: three of the GPU filler function (three seeds) and one of the system generator of each of configurations B (OpenSSL) and C (Windows, BCryptGenRandom).</t>
   </si>
   <si>
-    <t xml:space="preserve">S5_ConfigD — BenchmarkDotNet statistics of configuration D (laptop ASUS ROG Strix SCAR 18; Intel Core i9-14900HX, 32 threads; Intel UHD Graphics via OpenCL; NVIDIA GeForce RTX 4090 Laptop GPU via CUDA; Windows 11 Home 25H2; .NET 8.0.33; BenchmarkDotNet 0.15.8; ILGPU 1.5.3), every case of the six benchmark classes of the revision kit (measurement/laptop): break-even grid (3 processes x (5 warm-up + 30 measured iterations)), 10 MB formation, recovery, and recognition (1 x (3 + 15)), 100 MB full cycle and chunk size (1 x (2 + 10)). Times in milliseconds; CI = half-width of the 99.9% confidence interval of the mean (Student t, N - 1 degrees of freedom); N = measured iterations after the removal of upper outliers, pooled over the processes. Mean, CI, SD and SE are computed from the times of these iterations in the BenchmarkDotNet logs, as BenchmarkDotNet computes them; they agree with its reports, which give them rounded, and the manuscript uses them. Median, quartiles, extremes, allocation and collections are those of the reports. Process 1-3 = mean of the measured iterations of each process after the removal of upper outliers (WorkloadResult lines of the log).</t>
+    <t xml:space="preserve">S5_ConfigD — BenchmarkDotNet statistics of configuration D (laptop ASUS ROG Strix SCAR 18; Intel Core i9-14900HX, 32 threads; Intel UHD Graphics via OpenCL; NVIDIA GeForce RTX 4090 Laptop GPU via CUDA; Windows 11 Home 25H2; .NET 8.0.33; BenchmarkDotNet 0.15.8; ILGPU 1.5.3), every case of the six benchmark classes of the measurement kit of configuration D (measurement/laptop): break-even grid (3 processes x (5 warm-up + 30 measured iterations)), 10 MB formation, recovery, and recognition (1 x (3 + 15)), 100 MB full cycle and chunk size (1 x (2 + 10)). Times in milliseconds; CI = half-width of the 99.9% confidence interval of the mean (Student t, N - 1 degrees of freedom); N = measured iterations after the removal of upper outliers, pooled over the processes. Mean, CI, SD and SE are computed from the times of these iterations in the BenchmarkDotNet logs, as BenchmarkDotNet computes them; they agree with its reports, which give them rounded, and the manuscript uses them. Median, quartiles, extremes, allocation and collections are those of the reports. Process 1-3 = mean of the measured iterations of each process after the removal of upper outliers (WorkloadResult lines of the log).</t>
   </si>
   <si>
     <t xml:space="preserve">   Source: results/configuration_D of the repository (CSV reports and logs); analysis/config_d.py recomputes the tables of the manuscript and checks the means and N of the logs against the reports.</t>
@@ -694,7 +694,7 @@
     <t xml:space="preserve">LinearComplexity</t>
   </si>
   <si>
-    <t xml:space="preserve">Table S5. BenchmarkDotNet statistics of configuration D (all cases of the revision kit). Times in ms. Mean, CI, SD and SE computed from the iteration times of the BenchmarkDotNet logs (see README); CV = SD / Mean (formula). Process means from the logs; Process 2 and 3 empty for the classes run in one process.</t>
+    <t xml:space="preserve">Table S5. BenchmarkDotNet statistics of configuration D (all cases of the measurement kit of configuration D). Times in ms. Mean, CI, SD and SE computed from the iteration times of the BenchmarkDotNet logs (see README); CV = SD / Mean (formula). Process means from the logs; Process 2 and 3 empty for the classes run in one process.</t>
   </si>
   <si>
     <t xml:space="preserve">Class</t>

</xml_diff>